<commit_message>
feat: Basic Auth Middleware und env-Setup hinzugefügt
</commit_message>
<xml_diff>
--- a/app/public/Kurstransfer/Planungstabellen Excel/Kurstransfer-MS-Office.xlsx
+++ b/app/public/Kurstransfer/Planungstabellen Excel/Kurstransfer-MS-Office.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\temp\Kursplan-Projekt\app\public\Kurstransfer\Planungstabellen Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9276D202-3A43-46C0-B818-1EA62641F6D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{030A4412-1FEF-4B3D-ADC5-D0BDDFDBEB1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,6 +16,9 @@
     <sheet name="Terminplanung 2027" sheetId="1" r:id="rId1"/>
     <sheet name="Kurs_Definitionen" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Terminplanung 2027'!$A$1:$L$262</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -1581,7 +1584,9 @@
       </c>
       <c r="F26" s="6"/>
       <c r="G26" s="6"/>
-      <c r="H26" s="6"/>
+      <c r="H26" s="6" t="s">
+        <v>43</v>
+      </c>
       <c r="I26" s="6"/>
       <c r="J26" s="3" t="s">
         <v>21</v>
@@ -1609,9 +1614,6 @@
       </c>
       <c r="F27" s="6"/>
       <c r="G27" s="6"/>
-      <c r="H27" s="6" t="s">
-        <v>43</v>
-      </c>
       <c r="I27" s="6"/>
       <c r="J27" s="3" t="s">
         <v>21</v>
@@ -2151,7 +2153,9 @@
       </c>
       <c r="F45" s="6"/>
       <c r="G45" s="6"/>
-      <c r="H45" s="6"/>
+      <c r="H45" s="6" t="s">
+        <v>43</v>
+      </c>
       <c r="I45" s="6"/>
       <c r="J45" s="3" t="s">
         <v>21</v>
@@ -2209,9 +2213,6 @@
       </c>
       <c r="F47" s="6"/>
       <c r="G47" s="6"/>
-      <c r="H47" s="6" t="s">
-        <v>43</v>
-      </c>
       <c r="I47" s="6"/>
       <c r="J47" s="3" t="s">
         <v>21</v>
@@ -2773,7 +2774,9 @@
       </c>
       <c r="F66" s="6"/>
       <c r="G66" s="6"/>
-      <c r="H66" s="6"/>
+      <c r="H66" s="6" t="s">
+        <v>43</v>
+      </c>
       <c r="I66" s="6"/>
       <c r="J66" s="3" t="s">
         <v>21</v>
@@ -2801,9 +2804,6 @@
       </c>
       <c r="F67" s="6"/>
       <c r="G67" s="6"/>
-      <c r="H67" s="6" t="s">
-        <v>43</v>
-      </c>
       <c r="I67" s="6"/>
       <c r="J67" s="3" t="s">
         <v>21</v>
@@ -3981,7 +3981,9 @@
       </c>
       <c r="F108" s="11"/>
       <c r="G108" s="11"/>
-      <c r="H108" s="11"/>
+      <c r="H108" s="6" t="s">
+        <v>43</v>
+      </c>
       <c r="I108" s="11"/>
       <c r="J108" s="8" t="s">
         <v>21</v>
@@ -4099,9 +4101,6 @@
       </c>
       <c r="F112" s="6"/>
       <c r="G112" s="6"/>
-      <c r="H112" s="6" t="s">
-        <v>43</v>
-      </c>
       <c r="I112" s="6"/>
       <c r="J112" s="3" t="s">
         <v>21</v>
@@ -4641,7 +4640,9 @@
       </c>
       <c r="F130" s="6"/>
       <c r="G130" s="6"/>
-      <c r="H130" s="6"/>
+      <c r="H130" s="6" t="s">
+        <v>43</v>
+      </c>
       <c r="I130" s="6"/>
       <c r="J130" s="3" t="s">
         <v>21</v>
@@ -4699,9 +4700,6 @@
       </c>
       <c r="F132" s="6"/>
       <c r="G132" s="6"/>
-      <c r="H132" s="6" t="s">
-        <v>43</v>
-      </c>
       <c r="I132" s="6"/>
       <c r="J132" s="3" t="s">
         <v>21</v>
@@ -5793,7 +5791,9 @@
         <v>40</v>
       </c>
       <c r="G173" s="11"/>
-      <c r="H173" s="11"/>
+      <c r="H173" s="6" t="s">
+        <v>43</v>
+      </c>
       <c r="I173" s="11"/>
       <c r="J173" s="8" t="s">
         <v>21</v>
@@ -5909,9 +5909,6 @@
       </c>
       <c r="F177" s="6"/>
       <c r="G177" s="6"/>
-      <c r="H177" s="6" t="s">
-        <v>43</v>
-      </c>
       <c r="I177" s="6"/>
       <c r="J177" s="3" t="s">
         <v>21</v>
@@ -6419,7 +6416,9 @@
       </c>
       <c r="F194" s="6"/>
       <c r="G194" s="6"/>
-      <c r="H194" s="6"/>
+      <c r="H194" s="6" t="s">
+        <v>43</v>
+      </c>
       <c r="I194" s="6"/>
       <c r="J194" s="3" t="s">
         <v>21</v>
@@ -6509,9 +6508,6 @@
       </c>
       <c r="F197" s="6"/>
       <c r="G197" s="6"/>
-      <c r="H197" s="6" t="s">
-        <v>43</v>
-      </c>
       <c r="I197" s="6"/>
       <c r="J197" s="3" t="s">
         <v>21</v>
@@ -7081,7 +7077,9 @@
       </c>
       <c r="F216" s="6"/>
       <c r="G216" s="6"/>
-      <c r="H216" s="6"/>
+      <c r="H216" s="6" t="s">
+        <v>43</v>
+      </c>
       <c r="I216" s="6"/>
       <c r="J216" s="3" t="s">
         <v>21</v>
@@ -7109,9 +7107,6 @@
       </c>
       <c r="F217" s="6"/>
       <c r="G217" s="6"/>
-      <c r="H217" s="6" t="s">
-        <v>43</v>
-      </c>
       <c r="I217" s="6"/>
       <c r="J217" s="3" t="s">
         <v>21</v>
@@ -7647,7 +7642,9 @@
       </c>
       <c r="F235" s="6"/>
       <c r="G235" s="6"/>
-      <c r="H235" s="6"/>
+      <c r="H235" s="6" t="s">
+        <v>43</v>
+      </c>
       <c r="I235" s="6"/>
       <c r="J235" s="3" t="s">
         <v>21</v>
@@ -7705,9 +7702,6 @@
       </c>
       <c r="F237" s="6"/>
       <c r="G237" s="6"/>
-      <c r="H237" s="6" t="s">
-        <v>43</v>
-      </c>
       <c r="I237" s="6"/>
       <c r="J237" s="3" t="s">
         <v>21</v>
@@ -8410,6 +8404,7 @@
       <c r="L262" s="6"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:L262" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>